<commit_message>
Updated Oct 2026 schedule manually to adjust for Vijaydashmi
</commit_message>
<xml_diff>
--- a/schedule_2026_10.xlsx
+++ b/schedule_2026_10.xlsx
@@ -912,7 +912,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>16</v>
@@ -938,7 +938,7 @@
         <v>23</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1119,7 +1119,7 @@
         <v>13</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>16</v>
@@ -1142,10 +1142,10 @@
         <v>13</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1159,16 +1159,16 @@
         <v>19</v>
       </c>
       <c r="D22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="G22" s="3" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1191,7 +1191,7 @@
         <v>12</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>